<commit_message>
atualização dos dados de 1Q26
</commit_message>
<xml_diff>
--- a/analise_eua/semicondutores/amd/amd_indicators.xlsx
+++ b/analise_eua/semicondutores/amd/amd_indicators.xlsx
@@ -21,13 +21,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -46,13 +49,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -422,149 +436,149 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>P/L Damodaran</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>P/L</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>L/P</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Margem Líquida</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>P/VPA</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Valor de Mercado</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Dívida Bruta</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Caixa e Equivalentes</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/EBITDA</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/PL</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ROE</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ROIC</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>FCO</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>FCI</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>FCF</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Free Cash Flow</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Capex</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Net Capex</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>R&amp;D</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Adj Net Capex</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Working Capital</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Reinvestment Rate</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>FCFE</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>FCFF</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Buyback</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>2025</v>
       </c>
       <c r="B2" t="n">
@@ -653,7 +667,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
         <v>2024</v>
       </c>
       <c r="B3" t="n">
@@ -742,7 +756,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="1" t="n">
         <v>2023</v>
       </c>
       <c r="B4" t="n">
@@ -831,7 +845,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="1" t="n">
         <v>2022</v>
       </c>
       <c r="B5" t="n">
@@ -920,7 +934,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="1" t="n">
         <v>2021</v>
       </c>
       <c r="B6" t="n">
@@ -1009,7 +1023,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="1" t="n">
         <v>2020</v>
       </c>
       <c r="B7" t="n">
@@ -1098,7 +1112,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="1" t="n">
         <v>2019</v>
       </c>
       <c r="B8" t="n">
@@ -1187,7 +1201,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="1" t="n">
         <v>2018</v>
       </c>
       <c r="B9" t="n">
@@ -1276,7 +1290,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="1" t="n">
         <v>2017</v>
       </c>
       <c r="B10" t="n">
@@ -1375,1483 +1389,1572 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC16"/>
+  <dimension ref="A1:AC17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>P/L Damodaran</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>P/L</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>L/P</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Margem Líquida</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>P/VPA</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Valor de Mercado</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Dívida Bruta</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Caixa e Equivalentes</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/EBITDA</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/PL</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ROE</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ROIC</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>FCO</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>FCI</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>FCF</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Free Cash Flow</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Capex</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Net Capex</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>R&amp;D</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Adj Net Capex</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Working Capital</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Reinvestment Rate</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>FCFE</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>FCFF</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Buyback</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>45927</v>
+      <c r="A2" s="2" t="n">
+        <v>46109</v>
       </c>
       <c r="B2" t="n">
-        <v>211.64</v>
+        <v>239.91</v>
       </c>
       <c r="C2" t="n">
-        <v>72.88</v>
+        <v>78.54000000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>1.37</v>
+        <v>1.27</v>
       </c>
       <c r="E2" t="n">
-        <v>1462</v>
+        <v>1682</v>
       </c>
       <c r="F2" t="n">
-        <v>13.44</v>
+        <v>13.49</v>
       </c>
       <c r="G2" t="n">
-        <v>4.33</v>
+        <v>5.15</v>
       </c>
       <c r="H2" t="n">
-        <v>263070540</v>
+        <v>331794330</v>
       </c>
       <c r="I2" t="n">
-        <v>2997</v>
+        <v>3871</v>
       </c>
       <c r="J2" t="n">
-        <v>7243</v>
+        <v>12347</v>
       </c>
       <c r="K2" t="n">
-        <v>-4246</v>
+        <v>-8476</v>
       </c>
       <c r="L2" t="n">
-        <v>-1.07</v>
+        <v>-2.03</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.13</v>
       </c>
       <c r="N2" t="n">
-        <v>67.2</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="O2" t="n">
-        <v>5.91</v>
+        <v>6.53</v>
       </c>
       <c r="P2" t="n">
-        <v>5.1</v>
+        <v>5.47</v>
       </c>
       <c r="Q2" t="n">
-        <v>2159</v>
+        <v>2955</v>
       </c>
       <c r="R2" t="n">
-        <v>-1337</v>
+        <v>-2565</v>
       </c>
       <c r="S2" t="n">
-        <v>-450</v>
+        <v>-350</v>
       </c>
       <c r="T2" t="n">
-        <v>1901</v>
+        <v>2566</v>
       </c>
       <c r="U2" t="n">
-        <v>258</v>
+        <v>389</v>
       </c>
       <c r="V2" t="n">
-        <v>-428</v>
+        <v>379</v>
       </c>
       <c r="W2" t="n">
-        <v>2139</v>
+        <v>2397</v>
       </c>
       <c r="X2" t="n">
-        <v>6969</v>
+        <v>8537</v>
       </c>
       <c r="Y2" t="n">
-        <v>15300</v>
+        <v>18122</v>
       </c>
       <c r="Z2" t="n">
-        <v>229.44</v>
+        <v>218.3</v>
       </c>
       <c r="AA2" t="n">
-        <v>5024</v>
+        <v>5696</v>
       </c>
       <c r="AB2" t="n">
-        <v>2294</v>
+        <v>2909</v>
       </c>
       <c r="AC2" t="n">
-        <v>89</v>
+        <v>221</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>45836</v>
+      <c r="A3" s="2" t="n">
+        <v>45927</v>
       </c>
       <c r="B3" t="n">
-        <v>264.11</v>
+        <v>211.64</v>
       </c>
       <c r="C3" t="n">
-        <v>87.59</v>
+        <v>72.88</v>
       </c>
       <c r="D3" t="n">
-        <v>1.14</v>
+        <v>1.37</v>
       </c>
       <c r="E3" t="n">
-        <v>55</v>
+        <v>1462</v>
       </c>
       <c r="F3" t="n">
-        <v>11.35</v>
+        <v>13.44</v>
       </c>
       <c r="G3" t="n">
-        <v>3.86</v>
+        <v>4.33</v>
       </c>
       <c r="H3" t="n">
-        <v>230303700</v>
+        <v>263070540</v>
       </c>
       <c r="I3" t="n">
-        <v>3886</v>
+        <v>3870</v>
       </c>
       <c r="J3" t="n">
-        <v>5867</v>
+        <v>7243</v>
       </c>
       <c r="K3" t="n">
-        <v>-1981</v>
+        <v>-3373</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.85</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.03</v>
+        <v>-0.06</v>
       </c>
       <c r="N3" t="n">
-        <v>65.36</v>
+        <v>66.98</v>
       </c>
       <c r="O3" t="n">
-        <v>4.39</v>
+        <v>5.91</v>
       </c>
       <c r="P3" t="n">
-        <v>3.72</v>
+        <v>5.03</v>
       </c>
       <c r="Q3" t="n">
-        <v>2011</v>
+        <v>2159</v>
       </c>
       <c r="R3" t="n">
-        <v>-2298</v>
+        <v>-1337</v>
       </c>
       <c r="S3" t="n">
-        <v>-1319</v>
+        <v>-450</v>
       </c>
       <c r="T3" t="n">
-        <v>1729</v>
+        <v>1901</v>
       </c>
       <c r="U3" t="n">
-        <v>282</v>
+        <v>258</v>
       </c>
       <c r="V3" t="n">
-        <v>-1109</v>
+        <v>-428</v>
       </c>
       <c r="W3" t="n">
-        <v>1894</v>
+        <v>2139</v>
       </c>
       <c r="X3" t="n">
-        <v>5732</v>
+        <v>6969</v>
       </c>
       <c r="Y3" t="n">
-        <v>14676</v>
+        <v>15300</v>
       </c>
       <c r="Z3" t="n">
-        <v>224.43</v>
+        <v>229.44</v>
       </c>
       <c r="AA3" t="n">
-        <v>4898</v>
+        <v>5024</v>
       </c>
       <c r="AB3" t="n">
-        <v>-15560</v>
+        <v>2294</v>
       </c>
       <c r="AC3" t="n">
-        <v>478</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>45745</v>
+      <c r="A4" s="2" t="n">
+        <v>45836</v>
       </c>
       <c r="B4" t="n">
-        <v>234.75</v>
+        <v>264.11</v>
       </c>
       <c r="C4" t="n">
-        <v>88.56999999999999</v>
+        <v>87.59</v>
       </c>
       <c r="D4" t="n">
-        <v>1.13</v>
+        <v>1.14</v>
       </c>
       <c r="E4" t="n">
-        <v>981</v>
+        <v>55</v>
       </c>
       <c r="F4" t="n">
-        <v>9.529999999999999</v>
+        <v>11.35</v>
       </c>
       <c r="G4" t="n">
-        <v>2.88</v>
+        <v>3.86</v>
       </c>
       <c r="H4" t="n">
-        <v>166438800</v>
+        <v>230303700</v>
       </c>
       <c r="I4" t="n">
-        <v>4731</v>
+        <v>3886</v>
       </c>
       <c r="J4" t="n">
-        <v>7310</v>
+        <v>5867</v>
       </c>
       <c r="K4" t="n">
-        <v>-2579</v>
+        <v>-1981</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.6</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="M4" t="n">
-        <v>-0.04</v>
+        <v>-0.03</v>
       </c>
       <c r="N4" t="n">
-        <v>39.13</v>
+        <v>65.36</v>
       </c>
       <c r="O4" t="n">
-        <v>3.23</v>
+        <v>4.39</v>
       </c>
       <c r="P4" t="n">
-        <v>2.79</v>
+        <v>3.72</v>
       </c>
       <c r="Q4" t="n">
-        <v>939</v>
+        <v>2011</v>
       </c>
       <c r="R4" t="n">
-        <v>-357</v>
+        <v>-2298</v>
       </c>
       <c r="S4" t="n">
-        <v>1666</v>
+        <v>-1319</v>
       </c>
       <c r="T4" t="n">
-        <v>727</v>
+        <v>1729</v>
       </c>
       <c r="U4" t="n">
-        <v>212</v>
+        <v>282</v>
       </c>
       <c r="V4" t="n">
-        <v>-1844</v>
+        <v>-1109</v>
       </c>
       <c r="W4" t="n">
-        <v>1728</v>
+        <v>1894</v>
       </c>
       <c r="X4" t="n">
-        <v>4628</v>
+        <v>5732</v>
       </c>
       <c r="Y4" t="n">
-        <v>13892</v>
+        <v>14676</v>
       </c>
       <c r="Z4" t="n">
-        <v>316.74</v>
+        <v>224.43</v>
       </c>
       <c r="AA4" t="n">
-        <v>3541</v>
+        <v>4898</v>
       </c>
       <c r="AB4" t="n">
-        <v>2490</v>
+        <v>-15560</v>
       </c>
       <c r="AC4" t="n">
-        <v>749</v>
+        <v>478</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>45563</v>
+      <c r="A5" s="2" t="n">
+        <v>45745</v>
       </c>
       <c r="B5" t="n">
-        <v>344.76</v>
+        <v>234.75</v>
       </c>
       <c r="C5" t="n">
-        <v>180.31</v>
+        <v>88.56999999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>0.55</v>
+        <v>1.13</v>
       </c>
       <c r="E5" t="n">
-        <v>1480</v>
+        <v>981</v>
       </c>
       <c r="F5" t="n">
-        <v>11.31</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>4.66</v>
+        <v>2.88</v>
       </c>
       <c r="H5" t="n">
-        <v>265809600</v>
+        <v>166438800</v>
       </c>
       <c r="I5" t="n">
-        <v>2238</v>
+        <v>4731</v>
       </c>
       <c r="J5" t="n">
-        <v>4544</v>
+        <v>7310</v>
       </c>
       <c r="K5" t="n">
-        <v>-2306</v>
+        <v>-2579</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.53</v>
+        <v>-0.6</v>
       </c>
       <c r="M5" t="n">
         <v>-0.04</v>
       </c>
       <c r="N5" t="n">
-        <v>61.14</v>
+        <v>39.13</v>
       </c>
       <c r="O5" t="n">
-        <v>2.56</v>
+        <v>3.23</v>
       </c>
       <c r="P5" t="n">
-        <v>2.25</v>
+        <v>2.79</v>
       </c>
       <c r="Q5" t="n">
-        <v>628</v>
+        <v>939</v>
       </c>
       <c r="R5" t="n">
-        <v>-138</v>
+        <v>-357</v>
       </c>
       <c r="S5" t="n">
-        <v>-706</v>
+        <v>1666</v>
       </c>
       <c r="T5" t="n">
-        <v>496</v>
+        <v>727</v>
       </c>
       <c r="U5" t="n">
-        <v>132</v>
+        <v>212</v>
       </c>
       <c r="V5" t="n">
-        <v>-2580</v>
+        <v>-1844</v>
       </c>
       <c r="W5" t="n">
-        <v>1636</v>
+        <v>1728</v>
       </c>
       <c r="X5" t="n">
-        <v>3671</v>
+        <v>4628</v>
       </c>
       <c r="Y5" t="n">
-        <v>11235</v>
+        <v>13892</v>
       </c>
       <c r="Z5" t="n">
-        <v>371.28</v>
+        <v>316.74</v>
       </c>
       <c r="AA5" t="n">
-        <v>2021</v>
+        <v>3541</v>
       </c>
       <c r="AB5" t="n">
-        <v>2566</v>
+        <v>2490</v>
       </c>
       <c r="AC5" t="n">
-        <v>250</v>
+        <v>749</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>45472</v>
+      <c r="A6" s="2" t="n">
+        <v>45563</v>
       </c>
       <c r="B6" t="n">
-        <v>990.4</v>
+        <v>344.76</v>
       </c>
       <c r="C6" t="n">
-        <v>360.47</v>
+        <v>180.31</v>
       </c>
       <c r="D6" t="n">
-        <v>0.28</v>
+        <v>0.55</v>
       </c>
       <c r="E6" t="n">
-        <v>1038</v>
+        <v>1480</v>
       </c>
       <c r="F6" t="n">
-        <v>4.54</v>
+        <v>11.31</v>
       </c>
       <c r="G6" t="n">
-        <v>4.64</v>
+        <v>4.66</v>
       </c>
       <c r="H6" t="n">
-        <v>262455780</v>
+        <v>265809600</v>
       </c>
       <c r="I6" t="n">
-        <v>2245</v>
+        <v>2238</v>
       </c>
       <c r="J6" t="n">
-        <v>5340</v>
+        <v>4544</v>
       </c>
       <c r="K6" t="n">
-        <v>-3095</v>
+        <v>-2306</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.83</v>
+        <v>-0.53</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.05</v>
+        <v>-0.04</v>
       </c>
       <c r="N6" t="n">
-        <v>71.12</v>
+        <v>61.14</v>
       </c>
       <c r="O6" t="n">
-        <v>1.26</v>
+        <v>2.56</v>
       </c>
       <c r="P6" t="n">
-        <v>0.99</v>
+        <v>2.25</v>
       </c>
       <c r="Q6" t="n">
-        <v>593</v>
+        <v>628</v>
       </c>
       <c r="R6" t="n">
-        <v>386</v>
+        <v>-138</v>
       </c>
       <c r="S6" t="n">
-        <v>-1056</v>
+        <v>-706</v>
       </c>
       <c r="T6" t="n">
-        <v>439</v>
+        <v>496</v>
       </c>
       <c r="U6" t="n">
-        <v>154</v>
+        <v>132</v>
       </c>
       <c r="V6" t="n">
-        <v>-2680</v>
+        <v>-2580</v>
       </c>
       <c r="W6" t="n">
-        <v>1583</v>
+        <v>1636</v>
       </c>
       <c r="X6" t="n">
-        <v>3378</v>
+        <v>3671</v>
       </c>
       <c r="Y6" t="n">
-        <v>11270</v>
+        <v>11235</v>
       </c>
       <c r="Z6" t="n">
-        <v>717.53</v>
+        <v>371.28</v>
       </c>
       <c r="AA6" t="n">
-        <v>1846</v>
+        <v>2021</v>
       </c>
       <c r="AB6" t="n">
-        <v>2321</v>
+        <v>2566</v>
       </c>
       <c r="AC6" t="n">
-        <v>352</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>45381</v>
+      <c r="A7" s="2" t="n">
+        <v>45472</v>
       </c>
       <c r="B7" t="n">
-        <v>2372.78</v>
+        <v>990.4</v>
       </c>
       <c r="C7" t="n">
-        <v>902.45</v>
+        <v>360.47</v>
       </c>
       <c r="D7" t="n">
-        <v>0.11</v>
+        <v>0.28</v>
       </c>
       <c r="E7" t="n">
-        <v>820</v>
+        <v>1038</v>
       </c>
       <c r="F7" t="n">
-        <v>2.25</v>
+        <v>4.54</v>
       </c>
       <c r="G7" t="n">
-        <v>5.19</v>
+        <v>4.64</v>
       </c>
       <c r="H7" t="n">
-        <v>291852330</v>
+        <v>262455780</v>
       </c>
       <c r="I7" t="n">
-        <v>2998</v>
+        <v>2245</v>
       </c>
       <c r="J7" t="n">
-        <v>6035</v>
+        <v>5340</v>
       </c>
       <c r="K7" t="n">
-        <v>-3037</v>
+        <v>-3095</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.86</v>
+        <v>-0.83</v>
       </c>
       <c r="M7" t="n">
         <v>-0.05</v>
       </c>
       <c r="N7" t="n">
-        <v>83.47</v>
+        <v>71.12</v>
       </c>
       <c r="O7" t="n">
-        <v>0.55</v>
+        <v>1.26</v>
       </c>
       <c r="P7" t="n">
-        <v>0.33</v>
+        <v>0.99</v>
       </c>
       <c r="Q7" t="n">
-        <v>521</v>
+        <v>593</v>
       </c>
       <c r="R7" t="n">
-        <v>-135</v>
+        <v>386</v>
       </c>
       <c r="S7" t="n">
-        <v>-129</v>
+        <v>-1056</v>
       </c>
       <c r="T7" t="n">
-        <v>379</v>
+        <v>439</v>
       </c>
       <c r="U7" t="n">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="V7" t="n">
-        <v>-2889</v>
+        <v>-2680</v>
       </c>
       <c r="W7" t="n">
-        <v>1525</v>
+        <v>1583</v>
       </c>
       <c r="X7" t="n">
-        <v>2997</v>
+        <v>3378</v>
       </c>
       <c r="Y7" t="n">
-        <v>10610</v>
+        <v>11270</v>
       </c>
       <c r="Z7" t="n">
-        <v>1950.51</v>
+        <v>717.53</v>
       </c>
       <c r="AA7" t="n">
-        <v>2373</v>
+        <v>1846</v>
       </c>
       <c r="AB7" t="n">
-        <v>2158</v>
+        <v>2321</v>
       </c>
       <c r="AC7" t="n">
-        <v>4</v>
+        <v>352</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>45199</v>
+      <c r="A8" s="2" t="n">
+        <v>45381</v>
       </c>
       <c r="B8" t="n">
-        <v>555.71</v>
+        <v>2372.78</v>
       </c>
       <c r="C8" t="n">
-        <v>642.62</v>
+        <v>902.45</v>
       </c>
       <c r="D8" t="n">
-        <v>0.16</v>
+        <v>0.11</v>
       </c>
       <c r="E8" t="n">
-        <v>1047</v>
+        <v>820</v>
       </c>
       <c r="F8" t="n">
-        <v>5.16</v>
+        <v>2.25</v>
       </c>
       <c r="G8" t="n">
-        <v>3.02</v>
+        <v>5.19</v>
       </c>
       <c r="H8" t="n">
-        <v>166157120</v>
+        <v>291852330</v>
       </c>
       <c r="I8" t="n">
-        <v>2862</v>
+        <v>2998</v>
       </c>
       <c r="J8" t="n">
-        <v>5785</v>
+        <v>6035</v>
       </c>
       <c r="K8" t="n">
-        <v>-2923</v>
+        <v>-3037</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.77</v>
+        <v>-0.86</v>
       </c>
       <c r="M8" t="n">
         <v>-0.05</v>
       </c>
       <c r="N8" t="n">
-        <v>44.33</v>
+        <v>83.47</v>
       </c>
       <c r="O8" t="n">
-        <v>0.46</v>
+        <v>0.55</v>
       </c>
       <c r="P8" t="n">
-        <v>0.31</v>
+        <v>0.33</v>
       </c>
       <c r="Q8" t="n">
-        <v>421</v>
+        <v>521</v>
       </c>
       <c r="R8" t="n">
-        <v>102</v>
+        <v>-135</v>
       </c>
       <c r="S8" t="n">
-        <v>-803</v>
+        <v>-129</v>
       </c>
       <c r="T8" t="n">
-        <v>297</v>
+        <v>379</v>
       </c>
       <c r="U8" t="n">
-        <v>124</v>
+        <v>142</v>
       </c>
       <c r="V8" t="n">
-        <v>-3289</v>
+        <v>-2889</v>
       </c>
       <c r="W8" t="n">
-        <v>1507</v>
+        <v>1525</v>
       </c>
       <c r="X8" t="n">
-        <v>2351</v>
+        <v>2997</v>
       </c>
       <c r="Y8" t="n">
-        <v>9061</v>
+        <v>10610</v>
       </c>
       <c r="Z8" t="n">
-        <v>1903.91</v>
+        <v>1950.51</v>
       </c>
       <c r="AA8" t="n">
-        <v>2173</v>
+        <v>2373</v>
       </c>
       <c r="AB8" t="n">
-        <v>2226</v>
+        <v>2158</v>
       </c>
       <c r="AC8" t="n">
-        <v>511</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>45078</v>
+      <c r="A9" s="2" t="n">
+        <v>45199</v>
       </c>
       <c r="B9" t="n">
-        <v>6800.85</v>
+        <v>555.71</v>
       </c>
       <c r="C9" t="n">
-        <v>455.64</v>
+        <v>642.62</v>
       </c>
       <c r="D9" t="n">
-        <v>0.22</v>
+        <v>0.16</v>
       </c>
       <c r="E9" t="n">
-        <v>829</v>
+        <v>1047</v>
       </c>
       <c r="F9" t="n">
-        <v>0.5</v>
+        <v>5.16</v>
       </c>
       <c r="G9" t="n">
-        <v>3.33</v>
+        <v>3.02</v>
       </c>
       <c r="H9" t="n">
-        <v>183622920</v>
+        <v>166157120</v>
       </c>
       <c r="I9" t="n">
-        <v>2860</v>
+        <v>2862</v>
       </c>
       <c r="J9" t="n">
-        <v>6285</v>
+        <v>5785</v>
       </c>
       <c r="K9" t="n">
-        <v>-3425</v>
+        <v>-2923</v>
       </c>
       <c r="L9" t="n">
         <v>-0.77</v>
       </c>
       <c r="M9" t="n">
-        <v>-0.06</v>
+        <v>-0.05</v>
       </c>
       <c r="N9" t="n">
-        <v>41.82</v>
+        <v>44.33</v>
       </c>
       <c r="O9" t="n">
-        <v>0.73</v>
+        <v>0.46</v>
       </c>
       <c r="P9" t="n">
-        <v>0.67</v>
+        <v>0.31</v>
       </c>
       <c r="Q9" t="n">
-        <v>379</v>
+        <v>421</v>
       </c>
       <c r="R9" t="n">
-        <v>-438</v>
+        <v>102</v>
       </c>
       <c r="S9" t="n">
-        <v>75</v>
+        <v>-803</v>
       </c>
       <c r="T9" t="n">
-        <v>254</v>
+        <v>297</v>
       </c>
       <c r="U9" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="V9" t="n">
-        <v>-3638</v>
+        <v>-3289</v>
       </c>
       <c r="W9" t="n">
-        <v>1443</v>
+        <v>1507</v>
       </c>
       <c r="X9" t="n">
-        <v>1795</v>
+        <v>2351</v>
       </c>
       <c r="Y9" t="n">
-        <v>8933</v>
+        <v>9061</v>
       </c>
       <c r="Z9" t="n">
-        <v>683.25</v>
+        <v>1903.91</v>
       </c>
       <c r="AA9" t="n">
-        <v>2871</v>
+        <v>2173</v>
       </c>
       <c r="AB9" t="n">
-        <v>-337</v>
+        <v>2226</v>
       </c>
       <c r="AC9" t="n">
-        <v>0</v>
+        <v>511</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>44986</v>
+      <c r="A10" s="2" t="n">
+        <v>45078</v>
       </c>
       <c r="B10" t="n">
-        <v>-1135.93</v>
+        <v>6800.85</v>
       </c>
       <c r="C10" t="n">
-        <v>124.06</v>
+        <v>455.64</v>
       </c>
       <c r="D10" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.22</v>
       </c>
       <c r="E10" t="n">
-        <v>837</v>
+        <v>829</v>
       </c>
       <c r="F10" t="n">
-        <v>-2.6</v>
+        <v>0.5</v>
       </c>
       <c r="G10" t="n">
-        <v>2.89</v>
+        <v>3.33</v>
       </c>
       <c r="H10" t="n">
-        <v>157894110</v>
+        <v>183622920</v>
       </c>
       <c r="I10" t="n">
-        <v>2848</v>
+        <v>2860</v>
       </c>
       <c r="J10" t="n">
-        <v>5939</v>
+        <v>6285</v>
       </c>
       <c r="K10" t="n">
-        <v>-3091</v>
+        <v>-3425</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.59</v>
+        <v>-0.77</v>
       </c>
       <c r="M10" t="n">
         <v>-0.06</v>
       </c>
       <c r="N10" t="n">
-        <v>30.93</v>
+        <v>41.82</v>
       </c>
       <c r="O10" t="n">
-        <v>2.12</v>
+        <v>0.73</v>
       </c>
       <c r="P10" t="n">
-        <v>2.13</v>
+        <v>0.67</v>
       </c>
       <c r="Q10" t="n">
-        <v>486</v>
+        <v>379</v>
       </c>
       <c r="R10" t="n">
-        <v>-1237</v>
+        <v>-438</v>
       </c>
       <c r="S10" t="n">
-        <v>-259</v>
+        <v>75</v>
       </c>
       <c r="T10" t="n">
-        <v>328</v>
+        <v>254</v>
       </c>
       <c r="U10" t="n">
-        <v>158</v>
+        <v>125</v>
       </c>
       <c r="V10" t="n">
-        <v>-3452</v>
+        <v>-3638</v>
       </c>
       <c r="W10" t="n">
-        <v>1411</v>
+        <v>1443</v>
       </c>
       <c r="X10" t="n">
-        <v>1598</v>
+        <v>1795</v>
       </c>
       <c r="Y10" t="n">
-        <v>9081</v>
+        <v>8933</v>
       </c>
       <c r="Z10" t="n">
-        <v>187.49</v>
+        <v>683.25</v>
       </c>
       <c r="AA10" t="n">
-        <v>3605</v>
+        <v>2871</v>
       </c>
       <c r="AB10" t="n">
-        <v>4025</v>
+        <v>-337</v>
       </c>
       <c r="AC10" t="n">
-        <v>241</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>44828</v>
+      <c r="A11" s="2" t="n">
+        <v>44986</v>
       </c>
       <c r="B11" t="n">
-        <v>1550.4</v>
+        <v>-1135.93</v>
       </c>
       <c r="C11" t="n">
-        <v>38.63</v>
+        <v>124.06</v>
       </c>
       <c r="D11" t="n">
-        <v>2.59</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>1101</v>
+        <v>837</v>
       </c>
       <c r="F11" t="n">
-        <v>1.19</v>
+        <v>-2.6</v>
       </c>
       <c r="G11" t="n">
-        <v>1.88</v>
+        <v>2.89</v>
       </c>
       <c r="H11" t="n">
-        <v>102326400</v>
+        <v>157894110</v>
       </c>
       <c r="I11" t="n">
-        <v>2890</v>
+        <v>2848</v>
       </c>
       <c r="J11" t="n">
-        <v>5591</v>
+        <v>5939</v>
       </c>
       <c r="K11" t="n">
-        <v>-2701</v>
+        <v>-3091</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.5</v>
+        <v>-0.59</v>
       </c>
       <c r="M11" t="n">
-        <v>-0.05</v>
+        <v>-0.06</v>
       </c>
       <c r="N11" t="n">
-        <v>19.41</v>
+        <v>30.93</v>
       </c>
       <c r="O11" t="n">
-        <v>4.07</v>
+        <v>2.12</v>
       </c>
       <c r="P11" t="n">
-        <v>3.91</v>
+        <v>2.13</v>
       </c>
       <c r="Q11" t="n">
-        <v>965</v>
+        <v>486</v>
       </c>
       <c r="R11" t="n">
-        <v>-1298</v>
+        <v>-1237</v>
       </c>
       <c r="S11" t="n">
-        <v>-1233</v>
+        <v>-259</v>
       </c>
       <c r="T11" t="n">
-        <v>842</v>
+        <v>328</v>
       </c>
       <c r="U11" t="n">
-        <v>123</v>
+        <v>158</v>
       </c>
       <c r="V11" t="n">
-        <v>-2640</v>
+        <v>-3452</v>
       </c>
       <c r="W11" t="n">
-        <v>1279</v>
+        <v>1411</v>
       </c>
       <c r="X11" t="n">
-        <v>1764</v>
+        <v>1598</v>
       </c>
       <c r="Y11" t="n">
-        <v>7729</v>
+        <v>9081</v>
       </c>
       <c r="Z11" t="n">
-        <v>103.6</v>
+        <v>187.49</v>
       </c>
       <c r="AA11" t="n">
-        <v>3986</v>
+        <v>3605</v>
       </c>
       <c r="AB11" t="n">
-        <v>71</v>
+        <v>4025</v>
       </c>
       <c r="AC11" t="n">
-        <v>617</v>
+        <v>241</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>44737</v>
+      <c r="A12" s="2" t="n">
+        <v>44828</v>
       </c>
       <c r="B12" t="n">
-        <v>276.8</v>
+        <v>1550.4</v>
       </c>
       <c r="C12" t="n">
-        <v>35.08</v>
+        <v>38.63</v>
       </c>
       <c r="D12" t="n">
-        <v>2.85</v>
+        <v>2.59</v>
       </c>
       <c r="E12" t="n">
-        <v>1706</v>
+        <v>1101</v>
       </c>
       <c r="F12" t="n">
-        <v>6.82</v>
+        <v>1.19</v>
       </c>
       <c r="G12" t="n">
-        <v>2.24</v>
+        <v>1.88</v>
       </c>
       <c r="H12" t="n">
-        <v>123728460</v>
+        <v>102326400</v>
       </c>
       <c r="I12" t="n">
-        <v>3199</v>
+        <v>2890</v>
       </c>
       <c r="J12" t="n">
-        <v>5992</v>
+        <v>5591</v>
       </c>
       <c r="K12" t="n">
-        <v>-2793</v>
+        <v>-2701</v>
       </c>
       <c r="L12" t="n">
-        <v>-0.53</v>
+        <v>-0.5</v>
       </c>
       <c r="M12" t="n">
         <v>-0.05</v>
       </c>
       <c r="N12" t="n">
-        <v>24.15</v>
+        <v>19.41</v>
       </c>
       <c r="O12" t="n">
-        <v>5.19</v>
+        <v>4.07</v>
       </c>
       <c r="P12" t="n">
-        <v>4.96</v>
+        <v>3.91</v>
       </c>
       <c r="Q12" t="n">
-        <v>1038</v>
+        <v>965</v>
       </c>
       <c r="R12" t="n">
-        <v>-928</v>
+        <v>-1298</v>
       </c>
       <c r="S12" t="n">
-        <v>114</v>
+        <v>-1233</v>
       </c>
       <c r="T12" t="n">
-        <v>906</v>
+        <v>842</v>
       </c>
       <c r="U12" t="n">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="V12" t="n">
-        <v>-1631</v>
+        <v>-2640</v>
       </c>
       <c r="W12" t="n">
-        <v>1300</v>
+        <v>1279</v>
       </c>
       <c r="X12" t="n">
-        <v>2153</v>
+        <v>1764</v>
       </c>
       <c r="Y12" t="n">
-        <v>7939</v>
+        <v>7729</v>
       </c>
       <c r="Z12" t="n">
-        <v>109.16</v>
+        <v>103.6</v>
       </c>
       <c r="AA12" t="n">
-        <v>3491</v>
+        <v>3986</v>
       </c>
       <c r="AB12" t="n">
-        <v>3527</v>
+        <v>71</v>
       </c>
       <c r="AC12" t="n">
-        <v>921</v>
+        <v>617</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>44646</v>
+      <c r="A13" s="2" t="n">
+        <v>44737</v>
       </c>
       <c r="B13" t="n">
-        <v>193.78</v>
+        <v>276.8</v>
       </c>
       <c r="C13" t="n">
-        <v>46.33</v>
+        <v>35.08</v>
       </c>
       <c r="D13" t="n">
-        <v>2.16</v>
+        <v>2.85</v>
       </c>
       <c r="E13" t="n">
-        <v>1560</v>
+        <v>1706</v>
       </c>
       <c r="F13" t="n">
-        <v>13.35</v>
+        <v>6.82</v>
       </c>
       <c r="G13" t="n">
-        <v>2.75</v>
+        <v>2.24</v>
       </c>
       <c r="H13" t="n">
-        <v>152310620</v>
+        <v>123728460</v>
       </c>
       <c r="I13" t="n">
-        <v>2157</v>
+        <v>3199</v>
       </c>
       <c r="J13" t="n">
-        <v>6532</v>
+        <v>5992</v>
       </c>
       <c r="K13" t="n">
-        <v>-4375</v>
+        <v>-2793</v>
       </c>
       <c r="L13" t="n">
-        <v>-1.02</v>
+        <v>-0.53</v>
       </c>
       <c r="M13" t="n">
-        <v>-0.08</v>
+        <v>-0.05</v>
       </c>
       <c r="N13" t="n">
-        <v>36.52</v>
+        <v>24.15</v>
       </c>
       <c r="O13" t="n">
-        <v>5.37</v>
+        <v>5.19</v>
       </c>
       <c r="P13" t="n">
-        <v>5.21</v>
+        <v>4.96</v>
       </c>
       <c r="Q13" t="n">
-        <v>995</v>
+        <v>1038</v>
       </c>
       <c r="R13" t="n">
-        <v>3158</v>
+        <v>-928</v>
       </c>
       <c r="S13" t="n">
-        <v>-1948</v>
+        <v>114</v>
       </c>
       <c r="T13" t="n">
-        <v>924</v>
+        <v>906</v>
       </c>
       <c r="U13" t="n">
-        <v>71</v>
+        <v>132</v>
       </c>
       <c r="V13" t="n">
-        <v>-612</v>
+        <v>-1631</v>
       </c>
       <c r="W13" t="n">
-        <v>1060</v>
+        <v>1300</v>
       </c>
       <c r="X13" t="n">
-        <v>2482</v>
+        <v>2153</v>
       </c>
       <c r="Y13" t="n">
-        <v>7788</v>
+        <v>7939</v>
       </c>
       <c r="Z13" t="n">
-        <v>108.35</v>
+        <v>109.16</v>
       </c>
       <c r="AA13" t="n">
-        <v>2823</v>
+        <v>3491</v>
       </c>
       <c r="AB13" t="n">
-        <v>2813</v>
+        <v>3527</v>
       </c>
       <c r="AC13" t="n">
-        <v>1914</v>
+        <v>921</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>44464</v>
+      <c r="A14" s="2" t="n">
+        <v>44646</v>
       </c>
       <c r="B14" t="n">
-        <v>135.34</v>
+        <v>193.78</v>
       </c>
       <c r="C14" t="n">
-        <v>48.31</v>
+        <v>46.33</v>
       </c>
       <c r="D14" t="n">
-        <v>2.07</v>
+        <v>2.16</v>
       </c>
       <c r="E14" t="n">
-        <v>1045</v>
+        <v>1560</v>
       </c>
       <c r="F14" t="n">
-        <v>21.4</v>
+        <v>13.35</v>
       </c>
       <c r="G14" t="n">
-        <v>17.5</v>
+        <v>2.75</v>
       </c>
       <c r="H14" t="n">
-        <v>124920600</v>
+        <v>152310620</v>
       </c>
       <c r="I14" t="n">
-        <v>582</v>
+        <v>2157</v>
       </c>
       <c r="J14" t="n">
-        <v>3608</v>
+        <v>6532</v>
       </c>
       <c r="K14" t="n">
-        <v>-3026</v>
+        <v>-4375</v>
       </c>
       <c r="L14" t="n">
-        <v>-0.93</v>
+        <v>-1.02</v>
       </c>
       <c r="M14" t="n">
-        <v>-0.42</v>
+        <v>-0.08</v>
       </c>
       <c r="N14" t="n">
-        <v>39.24</v>
+        <v>36.52</v>
       </c>
       <c r="O14" t="n">
-        <v>36.13</v>
+        <v>5.37</v>
       </c>
       <c r="P14" t="n">
-        <v>33.61</v>
+        <v>5.21</v>
       </c>
       <c r="Q14" t="n">
-        <v>849</v>
+        <v>995</v>
       </c>
       <c r="R14" t="n">
-        <v>-83</v>
+        <v>3158</v>
       </c>
       <c r="S14" t="n">
-        <v>-949</v>
+        <v>-1948</v>
       </c>
       <c r="T14" t="n">
-        <v>764</v>
+        <v>924</v>
       </c>
       <c r="U14" t="n">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="V14" t="n">
-        <v>-82</v>
+        <v>-612</v>
       </c>
       <c r="W14" t="n">
-        <v>765</v>
+        <v>1060</v>
       </c>
       <c r="X14" t="n">
-        <v>2460</v>
+        <v>2482</v>
       </c>
       <c r="Y14" t="n">
-        <v>4424</v>
+        <v>7788</v>
       </c>
       <c r="Z14" t="n">
-        <v>103.55</v>
+        <v>108.35</v>
       </c>
       <c r="AA14" t="n">
-        <v>2234</v>
+        <v>2823</v>
       </c>
       <c r="AB14" t="n">
-        <v>2510</v>
+        <v>2813</v>
       </c>
       <c r="AC14" t="n">
-        <v>748</v>
+        <v>1914</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>44373</v>
+      <c r="A15" s="2" t="n">
+        <v>44464</v>
       </c>
       <c r="B15" t="n">
-        <v>160.87</v>
+        <v>135.34</v>
       </c>
       <c r="C15" t="n">
-        <v>62.62</v>
+        <v>48.31</v>
       </c>
       <c r="D15" t="n">
-        <v>1.6</v>
+        <v>2.07</v>
       </c>
       <c r="E15" t="n">
-        <v>928</v>
+        <v>1045</v>
       </c>
       <c r="F15" t="n">
-        <v>18.44</v>
+        <v>21.4</v>
       </c>
       <c r="G15" t="n">
-        <v>16.17</v>
+        <v>17.5</v>
       </c>
       <c r="H15" t="n">
-        <v>114218880</v>
+        <v>124920600</v>
       </c>
       <c r="I15" t="n">
-        <v>553</v>
+        <v>582</v>
       </c>
       <c r="J15" t="n">
-        <v>3793</v>
+        <v>3608</v>
       </c>
       <c r="K15" t="n">
-        <v>-3240</v>
+        <v>-3026</v>
       </c>
       <c r="L15" t="n">
-        <v>-1.32</v>
+        <v>-0.93</v>
       </c>
       <c r="M15" t="n">
-        <v>-0.46</v>
+        <v>-0.42</v>
       </c>
       <c r="N15" t="n">
-        <v>47.73</v>
+        <v>39.24</v>
       </c>
       <c r="O15" t="n">
-        <v>25.65</v>
+        <v>36.13</v>
       </c>
       <c r="P15" t="n">
-        <v>24.9</v>
+        <v>33.61</v>
       </c>
       <c r="Q15" t="n">
-        <v>952</v>
+        <v>849</v>
       </c>
       <c r="R15" t="n">
-        <v>119</v>
+        <v>-83</v>
       </c>
       <c r="S15" t="n">
-        <v>-211</v>
+        <v>-949</v>
       </c>
       <c r="T15" t="n">
-        <v>888</v>
+        <v>764</v>
       </c>
       <c r="U15" t="n">
-        <v>64</v>
+        <v>85</v>
       </c>
       <c r="V15" t="n">
-        <v>-51</v>
+        <v>-82</v>
       </c>
       <c r="W15" t="n">
-        <v>659</v>
+        <v>765</v>
       </c>
       <c r="X15" t="n">
-        <v>2186</v>
+        <v>2460</v>
       </c>
       <c r="Y15" t="n">
-        <v>4926</v>
+        <v>4424</v>
       </c>
       <c r="Z15" t="n">
-        <v>113.28</v>
+        <v>103.55</v>
       </c>
       <c r="AA15" t="n">
-        <v>1700</v>
+        <v>2234</v>
       </c>
       <c r="AB15" t="n">
-        <v>1912</v>
+        <v>2510</v>
       </c>
       <c r="AC15" t="n">
-        <v>256</v>
+        <v>748</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
+        <v>44373</v>
+      </c>
+      <c r="B16" t="n">
+        <v>160.87</v>
+      </c>
+      <c r="C16" t="n">
+        <v>62.62</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E16" t="n">
+        <v>928</v>
+      </c>
+      <c r="F16" t="n">
+        <v>18.44</v>
+      </c>
+      <c r="G16" t="n">
+        <v>16.17</v>
+      </c>
+      <c r="H16" t="n">
+        <v>114218880</v>
+      </c>
+      <c r="I16" t="n">
+        <v>553</v>
+      </c>
+      <c r="J16" t="n">
+        <v>3793</v>
+      </c>
+      <c r="K16" t="n">
+        <v>-3240</v>
+      </c>
+      <c r="L16" t="n">
+        <v>-1.32</v>
+      </c>
+      <c r="M16" t="n">
+        <v>-0.46</v>
+      </c>
+      <c r="N16" t="n">
+        <v>47.73</v>
+      </c>
+      <c r="O16" t="n">
+        <v>25.65</v>
+      </c>
+      <c r="P16" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>952</v>
+      </c>
+      <c r="R16" t="n">
+        <v>119</v>
+      </c>
+      <c r="S16" t="n">
+        <v>-211</v>
+      </c>
+      <c r="T16" t="n">
+        <v>888</v>
+      </c>
+      <c r="U16" t="n">
+        <v>64</v>
+      </c>
+      <c r="V16" t="n">
+        <v>-51</v>
+      </c>
+      <c r="W16" t="n">
+        <v>659</v>
+      </c>
+      <c r="X16" t="n">
+        <v>2186</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>4926</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>113.28</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>1700</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>1912</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
         <v>44282</v>
       </c>
-      <c r="B16" t="n">
+      <c r="B17" t="n">
         <v>171.57</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C17" t="n">
         <v>74.06</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D17" t="n">
         <v>1.35</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E17" t="n">
         <v>757</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F17" t="n">
         <v>16.11</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G17" t="n">
         <v>14.7</v>
       </c>
-      <c r="H16" t="n">
+      <c r="H17" t="n">
         <v>95220500</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I17" t="n">
         <v>551</v>
       </c>
-      <c r="J16" t="n">
+      <c r="J17" t="n">
         <v>3116</v>
       </c>
-      <c r="K16" t="n">
+      <c r="K17" t="n">
         <v>-2565</v>
       </c>
-      <c r="L16" t="n">
+      <c r="L17" t="n">
         <v>-1.44</v>
       </c>
-      <c r="M16" t="n">
+      <c r="M17" t="n">
         <v>-0.4</v>
       </c>
-      <c r="N16" t="n">
+      <c r="N17" t="n">
         <v>55</v>
       </c>
-      <c r="O16" t="n">
+      <c r="O17" t="n">
         <v>19.52</v>
       </c>
-      <c r="P16" t="n">
+      <c r="P17" t="n">
         <v>19.21</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="Q17" t="n">
         <v>898</v>
       </c>
-      <c r="R16" t="n">
+      <c r="R17" t="n">
         <v>-722</v>
       </c>
-      <c r="S16" t="n">
+      <c r="S17" t="n">
         <v>-8</v>
       </c>
-      <c r="T16" t="n">
+      <c r="T17" t="n">
         <v>832</v>
       </c>
-      <c r="U16" t="n">
+      <c r="U17" t="n">
         <v>66</v>
       </c>
-      <c r="V16" t="n">
+      <c r="V17" t="n">
         <v>-31</v>
       </c>
-      <c r="W16" t="n">
+      <c r="W17" t="n">
         <v>610</v>
       </c>
-      <c r="X16" t="n">
+      <c r="X17" t="n">
         <v>1989</v>
       </c>
-      <c r="Y16" t="n">
+      <c r="Y17" t="n">
         <v>4333</v>
       </c>
-      <c r="Z16" t="n">
+      <c r="Z17" t="n">
         <v>137.93</v>
       </c>
-      <c r="AA16" t="n">
+      <c r="AA17" t="n">
         <v>1222</v>
       </c>
-      <c r="AB16" t="n">
+      <c r="AB17" t="n">
         <v>1416</v>
       </c>
-      <c r="AC16" t="n">
+      <c r="AC17" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
atualizei os dados de 2Q26 da AMD
</commit_message>
<xml_diff>
--- a/analise_eua/semicondutores/amd/amd_indicators.xlsx
+++ b/analise_eua/semicondutores/amd/amd_indicators.xlsx
@@ -1389,7 +1389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC17"/>
+  <dimension ref="A1:AC18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1536,1425 +1536,1514 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46109</v>
+        <v>46200</v>
       </c>
       <c r="B2" t="n">
-        <v>239.91</v>
+        <v>412.73</v>
       </c>
       <c r="C2" t="n">
-        <v>78.54000000000001</v>
+        <v>163.18</v>
       </c>
       <c r="D2" t="n">
-        <v>1.27</v>
+        <v>0.61</v>
       </c>
       <c r="E2" t="n">
-        <v>1682</v>
+        <v>2211</v>
       </c>
       <c r="F2" t="n">
-        <v>13.49</v>
+        <v>19.91</v>
       </c>
       <c r="G2" t="n">
-        <v>5.15</v>
+        <v>14.1</v>
       </c>
       <c r="H2" t="n">
-        <v>331794330</v>
+        <v>948045120</v>
       </c>
       <c r="I2" t="n">
-        <v>3871</v>
+        <v>3401</v>
       </c>
       <c r="J2" t="n">
-        <v>12347</v>
+        <v>13111</v>
       </c>
       <c r="K2" t="n">
-        <v>-8476</v>
+        <v>-9710</v>
       </c>
       <c r="L2" t="n">
-        <v>-2.03</v>
+        <v>-1.79</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.13</v>
+        <v>-0.14</v>
       </c>
       <c r="N2" t="n">
-        <v>81.40000000000001</v>
+        <v>177.03</v>
       </c>
       <c r="O2" t="n">
-        <v>6.53</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="P2" t="n">
-        <v>5.47</v>
+        <v>6.79</v>
       </c>
       <c r="Q2" t="n">
-        <v>2955</v>
+        <v>2366</v>
       </c>
       <c r="R2" t="n">
-        <v>-2565</v>
+        <v>-2850</v>
       </c>
       <c r="S2" t="n">
-        <v>-350</v>
+        <v>-15</v>
       </c>
       <c r="T2" t="n">
-        <v>2566</v>
+        <v>1558</v>
       </c>
       <c r="U2" t="n">
-        <v>389</v>
+        <v>808</v>
       </c>
       <c r="V2" t="n">
-        <v>379</v>
+        <v>929</v>
       </c>
       <c r="W2" t="n">
-        <v>2397</v>
+        <v>2528</v>
       </c>
       <c r="X2" t="n">
-        <v>8537</v>
+        <v>9887</v>
       </c>
       <c r="Y2" t="n">
-        <v>18122</v>
+        <v>19441</v>
       </c>
       <c r="Z2" t="n">
-        <v>218.3</v>
+        <v>222.07</v>
       </c>
       <c r="AA2" t="n">
-        <v>5696</v>
+        <v>4106</v>
       </c>
       <c r="AB2" t="n">
-        <v>2909</v>
+        <v>2461</v>
       </c>
       <c r="AC2" t="n">
-        <v>221</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45927</v>
+        <v>46109</v>
       </c>
       <c r="B3" t="n">
-        <v>211.64</v>
+        <v>239.91</v>
       </c>
       <c r="C3" t="n">
-        <v>72.88</v>
+        <v>78.54000000000001</v>
       </c>
       <c r="D3" t="n">
-        <v>1.37</v>
+        <v>1.27</v>
       </c>
       <c r="E3" t="n">
-        <v>1462</v>
+        <v>1682</v>
       </c>
       <c r="F3" t="n">
-        <v>13.44</v>
+        <v>13.49</v>
       </c>
       <c r="G3" t="n">
-        <v>4.33</v>
+        <v>5.15</v>
       </c>
       <c r="H3" t="n">
-        <v>263070540</v>
+        <v>331794330</v>
       </c>
       <c r="I3" t="n">
-        <v>3870</v>
+        <v>3871</v>
       </c>
       <c r="J3" t="n">
-        <v>7243</v>
+        <v>12347</v>
       </c>
       <c r="K3" t="n">
-        <v>-3373</v>
+        <v>-8476</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.85</v>
+        <v>-2.03</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.06</v>
+        <v>-0.13</v>
       </c>
       <c r="N3" t="n">
-        <v>66.98</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="O3" t="n">
-        <v>5.91</v>
+        <v>6.53</v>
       </c>
       <c r="P3" t="n">
-        <v>5.03</v>
+        <v>5.47</v>
       </c>
       <c r="Q3" t="n">
-        <v>2159</v>
+        <v>2955</v>
       </c>
       <c r="R3" t="n">
-        <v>-1337</v>
+        <v>-2565</v>
       </c>
       <c r="S3" t="n">
-        <v>-450</v>
+        <v>-350</v>
       </c>
       <c r="T3" t="n">
-        <v>1901</v>
+        <v>2566</v>
       </c>
       <c r="U3" t="n">
-        <v>258</v>
+        <v>389</v>
       </c>
       <c r="V3" t="n">
-        <v>-428</v>
+        <v>379</v>
       </c>
       <c r="W3" t="n">
-        <v>2139</v>
+        <v>2397</v>
       </c>
       <c r="X3" t="n">
-        <v>6969</v>
+        <v>8537</v>
       </c>
       <c r="Y3" t="n">
-        <v>15300</v>
+        <v>18122</v>
       </c>
       <c r="Z3" t="n">
-        <v>229.44</v>
+        <v>218.3</v>
       </c>
       <c r="AA3" t="n">
-        <v>5024</v>
+        <v>5696</v>
       </c>
       <c r="AB3" t="n">
-        <v>2294</v>
+        <v>2909</v>
       </c>
       <c r="AC3" t="n">
-        <v>89</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45836</v>
+        <v>45927</v>
       </c>
       <c r="B4" t="n">
-        <v>264.11</v>
+        <v>211.64</v>
       </c>
       <c r="C4" t="n">
-        <v>87.59</v>
+        <v>72.88</v>
       </c>
       <c r="D4" t="n">
-        <v>1.14</v>
+        <v>1.37</v>
       </c>
       <c r="E4" t="n">
-        <v>55</v>
+        <v>1462</v>
       </c>
       <c r="F4" t="n">
-        <v>11.35</v>
+        <v>13.44</v>
       </c>
       <c r="G4" t="n">
-        <v>3.86</v>
+        <v>4.33</v>
       </c>
       <c r="H4" t="n">
-        <v>230303700</v>
+        <v>263070540</v>
       </c>
       <c r="I4" t="n">
-        <v>3886</v>
+        <v>3870</v>
       </c>
       <c r="J4" t="n">
-        <v>5867</v>
+        <v>7243</v>
       </c>
       <c r="K4" t="n">
-        <v>-1981</v>
+        <v>-3373</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.85</v>
       </c>
       <c r="M4" t="n">
-        <v>-0.03</v>
+        <v>-0.06</v>
       </c>
       <c r="N4" t="n">
-        <v>65.36</v>
+        <v>66.98</v>
       </c>
       <c r="O4" t="n">
-        <v>4.39</v>
+        <v>5.91</v>
       </c>
       <c r="P4" t="n">
-        <v>3.72</v>
+        <v>5.03</v>
       </c>
       <c r="Q4" t="n">
-        <v>2011</v>
+        <v>2159</v>
       </c>
       <c r="R4" t="n">
-        <v>-2298</v>
+        <v>-1337</v>
       </c>
       <c r="S4" t="n">
-        <v>-1319</v>
+        <v>-450</v>
       </c>
       <c r="T4" t="n">
-        <v>1729</v>
+        <v>1901</v>
       </c>
       <c r="U4" t="n">
-        <v>282</v>
+        <v>258</v>
       </c>
       <c r="V4" t="n">
-        <v>-1109</v>
+        <v>-428</v>
       </c>
       <c r="W4" t="n">
-        <v>1894</v>
+        <v>2139</v>
       </c>
       <c r="X4" t="n">
-        <v>5732</v>
+        <v>6969</v>
       </c>
       <c r="Y4" t="n">
-        <v>14676</v>
+        <v>15300</v>
       </c>
       <c r="Z4" t="n">
-        <v>224.43</v>
+        <v>229.44</v>
       </c>
       <c r="AA4" t="n">
-        <v>4898</v>
+        <v>5024</v>
       </c>
       <c r="AB4" t="n">
-        <v>-15560</v>
+        <v>2294</v>
       </c>
       <c r="AC4" t="n">
-        <v>478</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45745</v>
+        <v>45836</v>
       </c>
       <c r="B5" t="n">
-        <v>234.75</v>
+        <v>264.11</v>
       </c>
       <c r="C5" t="n">
-        <v>88.56999999999999</v>
+        <v>87.59</v>
       </c>
       <c r="D5" t="n">
-        <v>1.13</v>
+        <v>1.14</v>
       </c>
       <c r="E5" t="n">
-        <v>981</v>
+        <v>55</v>
       </c>
       <c r="F5" t="n">
-        <v>9.529999999999999</v>
+        <v>11.35</v>
       </c>
       <c r="G5" t="n">
-        <v>2.88</v>
+        <v>3.86</v>
       </c>
       <c r="H5" t="n">
-        <v>166438800</v>
+        <v>230303700</v>
       </c>
       <c r="I5" t="n">
-        <v>4731</v>
+        <v>3886</v>
       </c>
       <c r="J5" t="n">
-        <v>7310</v>
+        <v>5867</v>
       </c>
       <c r="K5" t="n">
-        <v>-2579</v>
+        <v>-1981</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.6</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.04</v>
+        <v>-0.03</v>
       </c>
       <c r="N5" t="n">
-        <v>39.13</v>
+        <v>65.36</v>
       </c>
       <c r="O5" t="n">
-        <v>3.23</v>
+        <v>4.39</v>
       </c>
       <c r="P5" t="n">
-        <v>2.79</v>
+        <v>3.72</v>
       </c>
       <c r="Q5" t="n">
-        <v>939</v>
+        <v>2011</v>
       </c>
       <c r="R5" t="n">
-        <v>-357</v>
+        <v>-2298</v>
       </c>
       <c r="S5" t="n">
-        <v>1666</v>
+        <v>-1319</v>
       </c>
       <c r="T5" t="n">
-        <v>727</v>
+        <v>1729</v>
       </c>
       <c r="U5" t="n">
-        <v>212</v>
+        <v>282</v>
       </c>
       <c r="V5" t="n">
-        <v>-1844</v>
+        <v>-1109</v>
       </c>
       <c r="W5" t="n">
-        <v>1728</v>
+        <v>1894</v>
       </c>
       <c r="X5" t="n">
-        <v>4628</v>
+        <v>5732</v>
       </c>
       <c r="Y5" t="n">
-        <v>13892</v>
+        <v>14676</v>
       </c>
       <c r="Z5" t="n">
-        <v>316.74</v>
+        <v>224.43</v>
       </c>
       <c r="AA5" t="n">
-        <v>3541</v>
+        <v>4898</v>
       </c>
       <c r="AB5" t="n">
-        <v>2490</v>
+        <v>-15560</v>
       </c>
       <c r="AC5" t="n">
-        <v>749</v>
+        <v>478</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45563</v>
+        <v>45745</v>
       </c>
       <c r="B6" t="n">
-        <v>344.76</v>
+        <v>234.75</v>
       </c>
       <c r="C6" t="n">
-        <v>180.31</v>
+        <v>88.56999999999999</v>
       </c>
       <c r="D6" t="n">
-        <v>0.55</v>
+        <v>1.13</v>
       </c>
       <c r="E6" t="n">
-        <v>1480</v>
+        <v>981</v>
       </c>
       <c r="F6" t="n">
-        <v>11.31</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>4.66</v>
+        <v>2.88</v>
       </c>
       <c r="H6" t="n">
-        <v>265809600</v>
+        <v>166438800</v>
       </c>
       <c r="I6" t="n">
-        <v>2238</v>
+        <v>4731</v>
       </c>
       <c r="J6" t="n">
-        <v>4544</v>
+        <v>7310</v>
       </c>
       <c r="K6" t="n">
-        <v>-2306</v>
+        <v>-2579</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.53</v>
+        <v>-0.6</v>
       </c>
       <c r="M6" t="n">
         <v>-0.04</v>
       </c>
       <c r="N6" t="n">
-        <v>61.14</v>
+        <v>39.13</v>
       </c>
       <c r="O6" t="n">
-        <v>2.56</v>
+        <v>3.23</v>
       </c>
       <c r="P6" t="n">
-        <v>2.25</v>
+        <v>2.79</v>
       </c>
       <c r="Q6" t="n">
-        <v>628</v>
+        <v>939</v>
       </c>
       <c r="R6" t="n">
-        <v>-138</v>
+        <v>-357</v>
       </c>
       <c r="S6" t="n">
-        <v>-706</v>
+        <v>1666</v>
       </c>
       <c r="T6" t="n">
-        <v>496</v>
+        <v>727</v>
       </c>
       <c r="U6" t="n">
-        <v>132</v>
+        <v>212</v>
       </c>
       <c r="V6" t="n">
-        <v>-2580</v>
+        <v>-1844</v>
       </c>
       <c r="W6" t="n">
-        <v>1636</v>
+        <v>1728</v>
       </c>
       <c r="X6" t="n">
-        <v>3671</v>
+        <v>4628</v>
       </c>
       <c r="Y6" t="n">
-        <v>11235</v>
+        <v>13892</v>
       </c>
       <c r="Z6" t="n">
-        <v>371.28</v>
+        <v>316.74</v>
       </c>
       <c r="AA6" t="n">
-        <v>2021</v>
+        <v>3541</v>
       </c>
       <c r="AB6" t="n">
-        <v>2566</v>
+        <v>2490</v>
       </c>
       <c r="AC6" t="n">
-        <v>250</v>
+        <v>749</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45472</v>
+        <v>45563</v>
       </c>
       <c r="B7" t="n">
-        <v>990.4</v>
+        <v>344.76</v>
       </c>
       <c r="C7" t="n">
-        <v>360.47</v>
+        <v>180.31</v>
       </c>
       <c r="D7" t="n">
-        <v>0.28</v>
+        <v>0.55</v>
       </c>
       <c r="E7" t="n">
-        <v>1038</v>
+        <v>1480</v>
       </c>
       <c r="F7" t="n">
-        <v>4.54</v>
+        <v>11.31</v>
       </c>
       <c r="G7" t="n">
-        <v>4.64</v>
+        <v>4.66</v>
       </c>
       <c r="H7" t="n">
-        <v>262455780</v>
+        <v>265809600</v>
       </c>
       <c r="I7" t="n">
-        <v>2245</v>
+        <v>2238</v>
       </c>
       <c r="J7" t="n">
-        <v>5340</v>
+        <v>4544</v>
       </c>
       <c r="K7" t="n">
-        <v>-3095</v>
+        <v>-2306</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.83</v>
+        <v>-0.53</v>
       </c>
       <c r="M7" t="n">
-        <v>-0.05</v>
+        <v>-0.04</v>
       </c>
       <c r="N7" t="n">
-        <v>71.12</v>
+        <v>61.14</v>
       </c>
       <c r="O7" t="n">
-        <v>1.26</v>
+        <v>2.56</v>
       </c>
       <c r="P7" t="n">
-        <v>0.99</v>
+        <v>2.25</v>
       </c>
       <c r="Q7" t="n">
-        <v>593</v>
+        <v>628</v>
       </c>
       <c r="R7" t="n">
-        <v>386</v>
+        <v>-138</v>
       </c>
       <c r="S7" t="n">
-        <v>-1056</v>
+        <v>-706</v>
       </c>
       <c r="T7" t="n">
-        <v>439</v>
+        <v>496</v>
       </c>
       <c r="U7" t="n">
-        <v>154</v>
+        <v>132</v>
       </c>
       <c r="V7" t="n">
-        <v>-2680</v>
+        <v>-2580</v>
       </c>
       <c r="W7" t="n">
-        <v>1583</v>
+        <v>1636</v>
       </c>
       <c r="X7" t="n">
-        <v>3378</v>
+        <v>3671</v>
       </c>
       <c r="Y7" t="n">
-        <v>11270</v>
+        <v>11235</v>
       </c>
       <c r="Z7" t="n">
-        <v>717.53</v>
+        <v>371.28</v>
       </c>
       <c r="AA7" t="n">
-        <v>1846</v>
+        <v>2021</v>
       </c>
       <c r="AB7" t="n">
-        <v>2321</v>
+        <v>2566</v>
       </c>
       <c r="AC7" t="n">
-        <v>352</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45381</v>
+        <v>45472</v>
       </c>
       <c r="B8" t="n">
-        <v>2372.78</v>
+        <v>990.4</v>
       </c>
       <c r="C8" t="n">
-        <v>902.45</v>
+        <v>360.47</v>
       </c>
       <c r="D8" t="n">
-        <v>0.11</v>
+        <v>0.28</v>
       </c>
       <c r="E8" t="n">
-        <v>820</v>
+        <v>1038</v>
       </c>
       <c r="F8" t="n">
-        <v>2.25</v>
+        <v>4.54</v>
       </c>
       <c r="G8" t="n">
-        <v>5.19</v>
+        <v>4.64</v>
       </c>
       <c r="H8" t="n">
-        <v>291852330</v>
+        <v>262455780</v>
       </c>
       <c r="I8" t="n">
-        <v>2998</v>
+        <v>2245</v>
       </c>
       <c r="J8" t="n">
-        <v>6035</v>
+        <v>5340</v>
       </c>
       <c r="K8" t="n">
-        <v>-3037</v>
+        <v>-3095</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.86</v>
+        <v>-0.83</v>
       </c>
       <c r="M8" t="n">
         <v>-0.05</v>
       </c>
       <c r="N8" t="n">
-        <v>83.47</v>
+        <v>71.12</v>
       </c>
       <c r="O8" t="n">
-        <v>0.55</v>
+        <v>1.26</v>
       </c>
       <c r="P8" t="n">
-        <v>0.33</v>
+        <v>0.99</v>
       </c>
       <c r="Q8" t="n">
-        <v>521</v>
+        <v>593</v>
       </c>
       <c r="R8" t="n">
-        <v>-135</v>
+        <v>386</v>
       </c>
       <c r="S8" t="n">
-        <v>-129</v>
+        <v>-1056</v>
       </c>
       <c r="T8" t="n">
-        <v>379</v>
+        <v>439</v>
       </c>
       <c r="U8" t="n">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="V8" t="n">
-        <v>-2889</v>
+        <v>-2680</v>
       </c>
       <c r="W8" t="n">
-        <v>1525</v>
+        <v>1583</v>
       </c>
       <c r="X8" t="n">
-        <v>2997</v>
+        <v>3378</v>
       </c>
       <c r="Y8" t="n">
-        <v>10610</v>
+        <v>11270</v>
       </c>
       <c r="Z8" t="n">
-        <v>1950.51</v>
+        <v>717.53</v>
       </c>
       <c r="AA8" t="n">
-        <v>2373</v>
+        <v>1846</v>
       </c>
       <c r="AB8" t="n">
-        <v>2158</v>
+        <v>2321</v>
       </c>
       <c r="AC8" t="n">
-        <v>4</v>
+        <v>352</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45199</v>
+        <v>45381</v>
       </c>
       <c r="B9" t="n">
-        <v>555.71</v>
+        <v>2372.78</v>
       </c>
       <c r="C9" t="n">
-        <v>642.62</v>
+        <v>902.45</v>
       </c>
       <c r="D9" t="n">
-        <v>0.16</v>
+        <v>0.11</v>
       </c>
       <c r="E9" t="n">
-        <v>1047</v>
+        <v>820</v>
       </c>
       <c r="F9" t="n">
-        <v>5.16</v>
+        <v>2.25</v>
       </c>
       <c r="G9" t="n">
-        <v>3.02</v>
+        <v>5.19</v>
       </c>
       <c r="H9" t="n">
-        <v>166157120</v>
+        <v>291852330</v>
       </c>
       <c r="I9" t="n">
-        <v>2862</v>
+        <v>2998</v>
       </c>
       <c r="J9" t="n">
-        <v>5785</v>
+        <v>6035</v>
       </c>
       <c r="K9" t="n">
-        <v>-2923</v>
+        <v>-3037</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.77</v>
+        <v>-0.86</v>
       </c>
       <c r="M9" t="n">
         <v>-0.05</v>
       </c>
       <c r="N9" t="n">
-        <v>44.33</v>
+        <v>83.47</v>
       </c>
       <c r="O9" t="n">
-        <v>0.46</v>
+        <v>0.55</v>
       </c>
       <c r="P9" t="n">
-        <v>0.31</v>
+        <v>0.33</v>
       </c>
       <c r="Q9" t="n">
-        <v>421</v>
+        <v>521</v>
       </c>
       <c r="R9" t="n">
-        <v>102</v>
+        <v>-135</v>
       </c>
       <c r="S9" t="n">
-        <v>-803</v>
+        <v>-129</v>
       </c>
       <c r="T9" t="n">
-        <v>297</v>
+        <v>379</v>
       </c>
       <c r="U9" t="n">
-        <v>124</v>
+        <v>142</v>
       </c>
       <c r="V9" t="n">
-        <v>-3289</v>
+        <v>-2889</v>
       </c>
       <c r="W9" t="n">
-        <v>1507</v>
+        <v>1525</v>
       </c>
       <c r="X9" t="n">
-        <v>2351</v>
+        <v>2997</v>
       </c>
       <c r="Y9" t="n">
-        <v>9061</v>
+        <v>10610</v>
       </c>
       <c r="Z9" t="n">
-        <v>1903.91</v>
+        <v>1950.51</v>
       </c>
       <c r="AA9" t="n">
-        <v>2173</v>
+        <v>2373</v>
       </c>
       <c r="AB9" t="n">
-        <v>2226</v>
+        <v>2158</v>
       </c>
       <c r="AC9" t="n">
-        <v>511</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45078</v>
+        <v>45199</v>
       </c>
       <c r="B10" t="n">
-        <v>6800.85</v>
+        <v>555.71</v>
       </c>
       <c r="C10" t="n">
-        <v>455.64</v>
+        <v>642.62</v>
       </c>
       <c r="D10" t="n">
-        <v>0.22</v>
+        <v>0.16</v>
       </c>
       <c r="E10" t="n">
-        <v>829</v>
+        <v>1047</v>
       </c>
       <c r="F10" t="n">
-        <v>0.5</v>
+        <v>5.16</v>
       </c>
       <c r="G10" t="n">
-        <v>3.33</v>
+        <v>3.02</v>
       </c>
       <c r="H10" t="n">
-        <v>183622920</v>
+        <v>166157120</v>
       </c>
       <c r="I10" t="n">
-        <v>2860</v>
+        <v>2862</v>
       </c>
       <c r="J10" t="n">
-        <v>6285</v>
+        <v>5785</v>
       </c>
       <c r="K10" t="n">
-        <v>-3425</v>
+        <v>-2923</v>
       </c>
       <c r="L10" t="n">
         <v>-0.77</v>
       </c>
       <c r="M10" t="n">
-        <v>-0.06</v>
+        <v>-0.05</v>
       </c>
       <c r="N10" t="n">
-        <v>41.82</v>
+        <v>44.33</v>
       </c>
       <c r="O10" t="n">
-        <v>0.73</v>
+        <v>0.46</v>
       </c>
       <c r="P10" t="n">
-        <v>0.67</v>
+        <v>0.31</v>
       </c>
       <c r="Q10" t="n">
-        <v>379</v>
+        <v>421</v>
       </c>
       <c r="R10" t="n">
-        <v>-438</v>
+        <v>102</v>
       </c>
       <c r="S10" t="n">
-        <v>75</v>
+        <v>-803</v>
       </c>
       <c r="T10" t="n">
-        <v>254</v>
+        <v>297</v>
       </c>
       <c r="U10" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="V10" t="n">
-        <v>-3638</v>
+        <v>-3289</v>
       </c>
       <c r="W10" t="n">
-        <v>1443</v>
+        <v>1507</v>
       </c>
       <c r="X10" t="n">
-        <v>1795</v>
+        <v>2351</v>
       </c>
       <c r="Y10" t="n">
-        <v>8933</v>
+        <v>9061</v>
       </c>
       <c r="Z10" t="n">
-        <v>683.25</v>
+        <v>1903.91</v>
       </c>
       <c r="AA10" t="n">
-        <v>2871</v>
+        <v>2173</v>
       </c>
       <c r="AB10" t="n">
-        <v>-337</v>
+        <v>2226</v>
       </c>
       <c r="AC10" t="n">
-        <v>0</v>
+        <v>511</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>44986</v>
+        <v>45078</v>
       </c>
       <c r="B11" t="n">
-        <v>-1135.93</v>
+        <v>6800.85</v>
       </c>
       <c r="C11" t="n">
-        <v>124.06</v>
+        <v>455.64</v>
       </c>
       <c r="D11" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.22</v>
       </c>
       <c r="E11" t="n">
-        <v>837</v>
+        <v>829</v>
       </c>
       <c r="F11" t="n">
-        <v>-2.6</v>
+        <v>0.5</v>
       </c>
       <c r="G11" t="n">
-        <v>2.89</v>
+        <v>3.33</v>
       </c>
       <c r="H11" t="n">
-        <v>157894110</v>
+        <v>183622920</v>
       </c>
       <c r="I11" t="n">
-        <v>2848</v>
+        <v>2860</v>
       </c>
       <c r="J11" t="n">
-        <v>5939</v>
+        <v>6285</v>
       </c>
       <c r="K11" t="n">
-        <v>-3091</v>
+        <v>-3425</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.59</v>
+        <v>-0.77</v>
       </c>
       <c r="M11" t="n">
         <v>-0.06</v>
       </c>
       <c r="N11" t="n">
-        <v>30.93</v>
+        <v>41.82</v>
       </c>
       <c r="O11" t="n">
-        <v>2.12</v>
+        <v>0.73</v>
       </c>
       <c r="P11" t="n">
-        <v>2.13</v>
+        <v>0.67</v>
       </c>
       <c r="Q11" t="n">
-        <v>486</v>
+        <v>379</v>
       </c>
       <c r="R11" t="n">
-        <v>-1237</v>
+        <v>-438</v>
       </c>
       <c r="S11" t="n">
-        <v>-259</v>
+        <v>75</v>
       </c>
       <c r="T11" t="n">
-        <v>328</v>
+        <v>254</v>
       </c>
       <c r="U11" t="n">
-        <v>158</v>
+        <v>125</v>
       </c>
       <c r="V11" t="n">
-        <v>-3452</v>
+        <v>-3638</v>
       </c>
       <c r="W11" t="n">
-        <v>1411</v>
+        <v>1443</v>
       </c>
       <c r="X11" t="n">
-        <v>1598</v>
+        <v>1795</v>
       </c>
       <c r="Y11" t="n">
-        <v>9081</v>
+        <v>8933</v>
       </c>
       <c r="Z11" t="n">
-        <v>187.49</v>
+        <v>683.25</v>
       </c>
       <c r="AA11" t="n">
-        <v>3605</v>
+        <v>2871</v>
       </c>
       <c r="AB11" t="n">
-        <v>4025</v>
+        <v>-337</v>
       </c>
       <c r="AC11" t="n">
-        <v>241</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>44828</v>
+        <v>44986</v>
       </c>
       <c r="B12" t="n">
-        <v>1550.4</v>
+        <v>-1135.93</v>
       </c>
       <c r="C12" t="n">
-        <v>38.63</v>
+        <v>124.06</v>
       </c>
       <c r="D12" t="n">
-        <v>2.59</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>1101</v>
+        <v>837</v>
       </c>
       <c r="F12" t="n">
-        <v>1.19</v>
+        <v>-2.6</v>
       </c>
       <c r="G12" t="n">
-        <v>1.88</v>
+        <v>2.89</v>
       </c>
       <c r="H12" t="n">
-        <v>102326400</v>
+        <v>157894110</v>
       </c>
       <c r="I12" t="n">
-        <v>2890</v>
+        <v>2848</v>
       </c>
       <c r="J12" t="n">
-        <v>5591</v>
+        <v>5939</v>
       </c>
       <c r="K12" t="n">
-        <v>-2701</v>
+        <v>-3091</v>
       </c>
       <c r="L12" t="n">
-        <v>-0.5</v>
+        <v>-0.59</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.05</v>
+        <v>-0.06</v>
       </c>
       <c r="N12" t="n">
-        <v>19.41</v>
+        <v>30.93</v>
       </c>
       <c r="O12" t="n">
-        <v>4.07</v>
+        <v>2.12</v>
       </c>
       <c r="P12" t="n">
-        <v>3.91</v>
+        <v>2.13</v>
       </c>
       <c r="Q12" t="n">
-        <v>965</v>
+        <v>486</v>
       </c>
       <c r="R12" t="n">
-        <v>-1298</v>
+        <v>-1237</v>
       </c>
       <c r="S12" t="n">
-        <v>-1233</v>
+        <v>-259</v>
       </c>
       <c r="T12" t="n">
-        <v>842</v>
+        <v>328</v>
       </c>
       <c r="U12" t="n">
-        <v>123</v>
+        <v>158</v>
       </c>
       <c r="V12" t="n">
-        <v>-2640</v>
+        <v>-3452</v>
       </c>
       <c r="W12" t="n">
-        <v>1279</v>
+        <v>1411</v>
       </c>
       <c r="X12" t="n">
-        <v>1764</v>
+        <v>1598</v>
       </c>
       <c r="Y12" t="n">
-        <v>7729</v>
+        <v>9081</v>
       </c>
       <c r="Z12" t="n">
-        <v>103.6</v>
+        <v>187.49</v>
       </c>
       <c r="AA12" t="n">
-        <v>3986</v>
+        <v>3605</v>
       </c>
       <c r="AB12" t="n">
-        <v>71</v>
+        <v>4025</v>
       </c>
       <c r="AC12" t="n">
-        <v>617</v>
+        <v>241</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>44737</v>
+        <v>44828</v>
       </c>
       <c r="B13" t="n">
-        <v>276.8</v>
+        <v>1550.4</v>
       </c>
       <c r="C13" t="n">
-        <v>35.08</v>
+        <v>38.63</v>
       </c>
       <c r="D13" t="n">
-        <v>2.85</v>
+        <v>2.59</v>
       </c>
       <c r="E13" t="n">
-        <v>1706</v>
+        <v>1101</v>
       </c>
       <c r="F13" t="n">
-        <v>6.82</v>
+        <v>1.19</v>
       </c>
       <c r="G13" t="n">
-        <v>2.24</v>
+        <v>1.88</v>
       </c>
       <c r="H13" t="n">
-        <v>123728460</v>
+        <v>102326400</v>
       </c>
       <c r="I13" t="n">
-        <v>3199</v>
+        <v>2890</v>
       </c>
       <c r="J13" t="n">
-        <v>5992</v>
+        <v>5591</v>
       </c>
       <c r="K13" t="n">
-        <v>-2793</v>
+        <v>-2701</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.53</v>
+        <v>-0.5</v>
       </c>
       <c r="M13" t="n">
         <v>-0.05</v>
       </c>
       <c r="N13" t="n">
-        <v>24.15</v>
+        <v>19.41</v>
       </c>
       <c r="O13" t="n">
-        <v>5.19</v>
+        <v>4.07</v>
       </c>
       <c r="P13" t="n">
-        <v>4.96</v>
+        <v>3.91</v>
       </c>
       <c r="Q13" t="n">
-        <v>1038</v>
+        <v>965</v>
       </c>
       <c r="R13" t="n">
-        <v>-928</v>
+        <v>-1298</v>
       </c>
       <c r="S13" t="n">
-        <v>114</v>
+        <v>-1233</v>
       </c>
       <c r="T13" t="n">
-        <v>906</v>
+        <v>842</v>
       </c>
       <c r="U13" t="n">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="V13" t="n">
-        <v>-1631</v>
+        <v>-2640</v>
       </c>
       <c r="W13" t="n">
-        <v>1300</v>
+        <v>1279</v>
       </c>
       <c r="X13" t="n">
-        <v>2153</v>
+        <v>1764</v>
       </c>
       <c r="Y13" t="n">
-        <v>7939</v>
+        <v>7729</v>
       </c>
       <c r="Z13" t="n">
-        <v>109.16</v>
+        <v>103.6</v>
       </c>
       <c r="AA13" t="n">
-        <v>3491</v>
+        <v>3986</v>
       </c>
       <c r="AB13" t="n">
-        <v>3527</v>
+        <v>71</v>
       </c>
       <c r="AC13" t="n">
-        <v>921</v>
+        <v>617</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>44646</v>
+        <v>44737</v>
       </c>
       <c r="B14" t="n">
-        <v>193.78</v>
+        <v>276.8</v>
       </c>
       <c r="C14" t="n">
-        <v>46.33</v>
+        <v>35.08</v>
       </c>
       <c r="D14" t="n">
-        <v>2.16</v>
+        <v>2.85</v>
       </c>
       <c r="E14" t="n">
-        <v>1560</v>
+        <v>1706</v>
       </c>
       <c r="F14" t="n">
-        <v>13.35</v>
+        <v>6.82</v>
       </c>
       <c r="G14" t="n">
-        <v>2.75</v>
+        <v>2.24</v>
       </c>
       <c r="H14" t="n">
-        <v>152310620</v>
+        <v>123728460</v>
       </c>
       <c r="I14" t="n">
-        <v>2157</v>
+        <v>3199</v>
       </c>
       <c r="J14" t="n">
-        <v>6532</v>
+        <v>5992</v>
       </c>
       <c r="K14" t="n">
-        <v>-4375</v>
+        <v>-2793</v>
       </c>
       <c r="L14" t="n">
-        <v>-1.02</v>
+        <v>-0.53</v>
       </c>
       <c r="M14" t="n">
-        <v>-0.08</v>
+        <v>-0.05</v>
       </c>
       <c r="N14" t="n">
-        <v>36.52</v>
+        <v>24.15</v>
       </c>
       <c r="O14" t="n">
-        <v>5.37</v>
+        <v>5.19</v>
       </c>
       <c r="P14" t="n">
-        <v>5.21</v>
+        <v>4.96</v>
       </c>
       <c r="Q14" t="n">
-        <v>995</v>
+        <v>1038</v>
       </c>
       <c r="R14" t="n">
-        <v>3158</v>
+        <v>-928</v>
       </c>
       <c r="S14" t="n">
-        <v>-1948</v>
+        <v>114</v>
       </c>
       <c r="T14" t="n">
-        <v>924</v>
+        <v>906</v>
       </c>
       <c r="U14" t="n">
-        <v>71</v>
+        <v>132</v>
       </c>
       <c r="V14" t="n">
-        <v>-612</v>
+        <v>-1631</v>
       </c>
       <c r="W14" t="n">
-        <v>1060</v>
+        <v>1300</v>
       </c>
       <c r="X14" t="n">
-        <v>2482</v>
+        <v>2153</v>
       </c>
       <c r="Y14" t="n">
-        <v>7788</v>
+        <v>7939</v>
       </c>
       <c r="Z14" t="n">
-        <v>108.35</v>
+        <v>109.16</v>
       </c>
       <c r="AA14" t="n">
-        <v>2823</v>
+        <v>3491</v>
       </c>
       <c r="AB14" t="n">
-        <v>2813</v>
+        <v>3527</v>
       </c>
       <c r="AC14" t="n">
-        <v>1914</v>
+        <v>921</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>44464</v>
+        <v>44646</v>
       </c>
       <c r="B15" t="n">
-        <v>135.34</v>
+        <v>193.78</v>
       </c>
       <c r="C15" t="n">
-        <v>48.31</v>
+        <v>46.33</v>
       </c>
       <c r="D15" t="n">
-        <v>2.07</v>
+        <v>2.16</v>
       </c>
       <c r="E15" t="n">
-        <v>1045</v>
+        <v>1560</v>
       </c>
       <c r="F15" t="n">
-        <v>21.4</v>
+        <v>13.35</v>
       </c>
       <c r="G15" t="n">
-        <v>17.5</v>
+        <v>2.75</v>
       </c>
       <c r="H15" t="n">
-        <v>124920600</v>
+        <v>152310620</v>
       </c>
       <c r="I15" t="n">
-        <v>582</v>
+        <v>2157</v>
       </c>
       <c r="J15" t="n">
-        <v>3608</v>
+        <v>6532</v>
       </c>
       <c r="K15" t="n">
-        <v>-3026</v>
+        <v>-4375</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.93</v>
+        <v>-1.02</v>
       </c>
       <c r="M15" t="n">
-        <v>-0.42</v>
+        <v>-0.08</v>
       </c>
       <c r="N15" t="n">
-        <v>39.24</v>
+        <v>36.52</v>
       </c>
       <c r="O15" t="n">
-        <v>36.13</v>
+        <v>5.37</v>
       </c>
       <c r="P15" t="n">
-        <v>33.61</v>
+        <v>5.21</v>
       </c>
       <c r="Q15" t="n">
-        <v>849</v>
+        <v>995</v>
       </c>
       <c r="R15" t="n">
-        <v>-83</v>
+        <v>3158</v>
       </c>
       <c r="S15" t="n">
-        <v>-949</v>
+        <v>-1948</v>
       </c>
       <c r="T15" t="n">
-        <v>764</v>
+        <v>924</v>
       </c>
       <c r="U15" t="n">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="V15" t="n">
-        <v>-82</v>
+        <v>-612</v>
       </c>
       <c r="W15" t="n">
-        <v>765</v>
+        <v>1060</v>
       </c>
       <c r="X15" t="n">
-        <v>2460</v>
+        <v>2482</v>
       </c>
       <c r="Y15" t="n">
-        <v>4424</v>
+        <v>7788</v>
       </c>
       <c r="Z15" t="n">
-        <v>103.55</v>
+        <v>108.35</v>
       </c>
       <c r="AA15" t="n">
-        <v>2234</v>
+        <v>2823</v>
       </c>
       <c r="AB15" t="n">
-        <v>2510</v>
+        <v>2813</v>
       </c>
       <c r="AC15" t="n">
-        <v>748</v>
+        <v>1914</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>44373</v>
+        <v>44464</v>
       </c>
       <c r="B16" t="n">
-        <v>160.87</v>
+        <v>135.34</v>
       </c>
       <c r="C16" t="n">
-        <v>62.62</v>
+        <v>48.31</v>
       </c>
       <c r="D16" t="n">
-        <v>1.6</v>
+        <v>2.07</v>
       </c>
       <c r="E16" t="n">
-        <v>928</v>
+        <v>1045</v>
       </c>
       <c r="F16" t="n">
-        <v>18.44</v>
+        <v>21.4</v>
       </c>
       <c r="G16" t="n">
-        <v>16.17</v>
+        <v>17.5</v>
       </c>
       <c r="H16" t="n">
-        <v>114218880</v>
+        <v>124920600</v>
       </c>
       <c r="I16" t="n">
-        <v>553</v>
+        <v>582</v>
       </c>
       <c r="J16" t="n">
-        <v>3793</v>
+        <v>3608</v>
       </c>
       <c r="K16" t="n">
-        <v>-3240</v>
+        <v>-3026</v>
       </c>
       <c r="L16" t="n">
-        <v>-1.32</v>
+        <v>-0.93</v>
       </c>
       <c r="M16" t="n">
-        <v>-0.46</v>
+        <v>-0.42</v>
       </c>
       <c r="N16" t="n">
-        <v>47.73</v>
+        <v>39.24</v>
       </c>
       <c r="O16" t="n">
-        <v>25.65</v>
+        <v>36.13</v>
       </c>
       <c r="P16" t="n">
-        <v>24.9</v>
+        <v>33.61</v>
       </c>
       <c r="Q16" t="n">
-        <v>952</v>
+        <v>849</v>
       </c>
       <c r="R16" t="n">
-        <v>119</v>
+        <v>-83</v>
       </c>
       <c r="S16" t="n">
-        <v>-211</v>
+        <v>-949</v>
       </c>
       <c r="T16" t="n">
-        <v>888</v>
+        <v>764</v>
       </c>
       <c r="U16" t="n">
-        <v>64</v>
+        <v>85</v>
       </c>
       <c r="V16" t="n">
-        <v>-51</v>
+        <v>-82</v>
       </c>
       <c r="W16" t="n">
-        <v>659</v>
+        <v>765</v>
       </c>
       <c r="X16" t="n">
-        <v>2186</v>
+        <v>2460</v>
       </c>
       <c r="Y16" t="n">
-        <v>4926</v>
+        <v>4424</v>
       </c>
       <c r="Z16" t="n">
-        <v>113.28</v>
+        <v>103.55</v>
       </c>
       <c r="AA16" t="n">
-        <v>1700</v>
+        <v>2234</v>
       </c>
       <c r="AB16" t="n">
-        <v>1912</v>
+        <v>2510</v>
       </c>
       <c r="AC16" t="n">
-        <v>256</v>
+        <v>748</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
+        <v>44373</v>
+      </c>
+      <c r="B17" t="n">
+        <v>160.87</v>
+      </c>
+      <c r="C17" t="n">
+        <v>62.62</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E17" t="n">
+        <v>928</v>
+      </c>
+      <c r="F17" t="n">
+        <v>18.44</v>
+      </c>
+      <c r="G17" t="n">
+        <v>16.17</v>
+      </c>
+      <c r="H17" t="n">
+        <v>114218880</v>
+      </c>
+      <c r="I17" t="n">
+        <v>553</v>
+      </c>
+      <c r="J17" t="n">
+        <v>3793</v>
+      </c>
+      <c r="K17" t="n">
+        <v>-3240</v>
+      </c>
+      <c r="L17" t="n">
+        <v>-1.32</v>
+      </c>
+      <c r="M17" t="n">
+        <v>-0.46</v>
+      </c>
+      <c r="N17" t="n">
+        <v>47.73</v>
+      </c>
+      <c r="O17" t="n">
+        <v>25.65</v>
+      </c>
+      <c r="P17" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>952</v>
+      </c>
+      <c r="R17" t="n">
+        <v>119</v>
+      </c>
+      <c r="S17" t="n">
+        <v>-211</v>
+      </c>
+      <c r="T17" t="n">
+        <v>888</v>
+      </c>
+      <c r="U17" t="n">
+        <v>64</v>
+      </c>
+      <c r="V17" t="n">
+        <v>-51</v>
+      </c>
+      <c r="W17" t="n">
+        <v>659</v>
+      </c>
+      <c r="X17" t="n">
+        <v>2186</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>4926</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>113.28</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>1700</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>1912</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
         <v>44282</v>
       </c>
-      <c r="B17" t="n">
+      <c r="B18" t="n">
         <v>171.57</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C18" t="n">
         <v>74.06</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D18" t="n">
         <v>1.35</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E18" t="n">
         <v>757</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F18" t="n">
         <v>16.11</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G18" t="n">
         <v>14.7</v>
       </c>
-      <c r="H17" t="n">
+      <c r="H18" t="n">
         <v>95220500</v>
       </c>
-      <c r="I17" t="n">
+      <c r="I18" t="n">
         <v>551</v>
       </c>
-      <c r="J17" t="n">
+      <c r="J18" t="n">
         <v>3116</v>
       </c>
-      <c r="K17" t="n">
+      <c r="K18" t="n">
         <v>-2565</v>
       </c>
-      <c r="L17" t="n">
+      <c r="L18" t="n">
         <v>-1.44</v>
       </c>
-      <c r="M17" t="n">
+      <c r="M18" t="n">
         <v>-0.4</v>
       </c>
-      <c r="N17" t="n">
+      <c r="N18" t="n">
         <v>55</v>
       </c>
-      <c r="O17" t="n">
+      <c r="O18" t="n">
         <v>19.52</v>
       </c>
-      <c r="P17" t="n">
+      <c r="P18" t="n">
         <v>19.21</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="Q18" t="n">
         <v>898</v>
       </c>
-      <c r="R17" t="n">
+      <c r="R18" t="n">
         <v>-722</v>
       </c>
-      <c r="S17" t="n">
+      <c r="S18" t="n">
         <v>-8</v>
       </c>
-      <c r="T17" t="n">
+      <c r="T18" t="n">
         <v>832</v>
       </c>
-      <c r="U17" t="n">
+      <c r="U18" t="n">
         <v>66</v>
       </c>
-      <c r="V17" t="n">
+      <c r="V18" t="n">
         <v>-31</v>
       </c>
-      <c r="W17" t="n">
+      <c r="W18" t="n">
         <v>610</v>
       </c>
-      <c r="X17" t="n">
+      <c r="X18" t="n">
         <v>1989</v>
       </c>
-      <c r="Y17" t="n">
+      <c r="Y18" t="n">
         <v>4333</v>
       </c>
-      <c r="Z17" t="n">
+      <c r="Z18" t="n">
         <v>137.93</v>
       </c>
-      <c r="AA17" t="n">
+      <c r="AA18" t="n">
         <v>1222</v>
       </c>
-      <c r="AB17" t="n">
+      <c r="AB18" t="n">
         <v>1416</v>
       </c>
-      <c r="AC17" t="n">
+      <c r="AC18" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>